<commit_message>
After-build report and the impairment workbook updated for the second round: the chain complete to the ECL
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/compliance/IFRS9_Impairment_Compliance_Audit.xlsx
+++ b/docs/compliance/IFRS9_Impairment_Compliance_Audit.xlsx
@@ -2115,27 +2115,27 @@
       </c>
       <c r="C5" s="22" t="inlineStr">
         <is>
-          <t>The PD engine has not run on the clean install</t>
+          <t>The PD and LGD of the clean install are the bootstrap's, not MAIIC's</t>
         </is>
       </c>
       <c r="D5" s="22" t="inlineStr">
         <is>
-          <t>The transition-matrix PD runs from its screen and is not yet callable by the bootstrap; every PD is null and the ECL of the period is nil.</t>
+          <t>PdEngineService and LgdEngineService run the transition matrix and the cohort workout under the bootstrap label; no MAIIC reviewer has key-locked a matrix or an LGD calculation in the system.</t>
         </is>
       </c>
       <c r="E5" s="22" t="inlineStr">
         <is>
-          <t>No weighted ECL for a period; the scenario sensitivity reports zero loans with a PD.</t>
+          <t>The ECL of 8.33bn at August 2026 is a system figure awaiting review.</t>
         </is>
       </c>
       <c r="F5" s="22" t="inlineStr">
         <is>
-          <t>Lift the transition-matrix logic into a service the bootstrap calls (engine step 4), then run the ECL under the approved scenario set.</t>
+          <t>A reviewer key-locks the matrix and the LGD on their screens; the ECL is then re-run under the approved scenario set.</t>
         </is>
       </c>
       <c r="G5" s="22" t="inlineStr">
         <is>
-          <t>Dupleix</t>
+          <t>Dr Thom / the reviewer</t>
         </is>
       </c>
       <c r="H5" s="22" t="inlineStr">
@@ -2279,7 +2279,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-10-08 20:26:01 from maiic_ifrs9_bootstrap. The PASS/FAIL in column E is a formula on columns B and C, so it recomputes if a figure is typed over.</t>
+          <t>Generated 2026-10-08 20:35:55 from maiic_ifrs9_bootstrap. The PASS/FAIL in column E is a formula on columns B and C, so it recomputes if a figure is typed over.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
The Mega Farm screen; the method cards inline on the Governance Centre setting (spec v4 s.16, 14.7)
Financial Modelling / Mega Farm Programme: the programme's book by scheme
and by stage for a period, the governed scope, method and ceiling in
force with whether D30 is confirmed, each run with its basis or the
reason it was declined, and the Run action for the governed role. The
Governance Centre shows, on every option of fli_transmission_method, a
badge saying whether the method can be selected and the method card on
request: what it does, the formula, what it implies, its preconditions
checked live against the data, a worked example. The after-build report,
the impairment workbook, the register and the help centre are updated.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/compliance/IFRS9_Impairment_Compliance_Audit.xlsx
+++ b/docs/compliance/IFRS9_Impairment_Compliance_Audit.xlsx
@@ -1728,7 +1728,7 @@
       </c>
       <c r="H15" s="22" t="inlineStr">
         <is>
-          <t>Financial Modelling, Forward-Looking Model: /regression; fli:correlate; fli:method-cards (fli:method-cards; /fli/transmission-methods)</t>
+          <t>Financial Modelling, Forward-Looking Model: /regression; fli:correlate; fli:method-cards; Governance Centre, the cards inline on the setting: /eir-governance; fli:method-cards</t>
         </is>
       </c>
       <c r="I15" s="22" t="inlineStr"/>
@@ -1971,7 +1971,7 @@
       </c>
       <c r="H22" s="22" t="inlineStr">
         <is>
-          <t>Governance Centre: /eir-governance; Data Foundation, Loan Book (2025-11)</t>
+          <t>Financial Modelling, Mega Farm Programme: /megafarm; Governance Centre: /eir-governance</t>
         </is>
       </c>
       <c r="I22" s="22" t="inlineStr"/>
@@ -2279,7 +2279,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-10-08 21:18:14 from maiic_ifrs9_bootstrap. The PASS/FAIL in column E is a formula on columns B and C, so it recomputes if a figure is typed over.</t>
+          <t>Generated 2026-10-08 21:40:05 from maiic_ifrs9_bootstrap. The PASS/FAIL in column E is a formula on columns B and C, so it recomputes if a figure is typed over.</t>
         </is>
       </c>
     </row>

</xml_diff>